<commit_message>
After rechecking the data, some categories were modified
</commit_message>
<xml_diff>
--- a/data/labeled_data/2_Uncertain/2_uncertain.xlsx
+++ b/data/labeled_data/2_Uncertain/2_uncertain.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="26860" windowHeight="11480"/>
+    <workbookView windowWidth="13060" windowHeight="13660"/>
   </bookViews>
   <sheets>
     <sheet name="前50条视频审核" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1272" uniqueCount="551">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1282" uniqueCount="557">
   <si>
     <t>ID</t>
   </si>
@@ -1667,6 +1667,24 @@
   </si>
   <si>
     <t>C0616</t>
+  </si>
+  <si>
+    <t>C0173</t>
+  </si>
+  <si>
+    <t>目标没有被遮挡并且在结束时出现了第二个目标</t>
+  </si>
+  <si>
+    <t>单个球体→两个球体</t>
+  </si>
+  <si>
+    <t>C0449</t>
+  </si>
+  <si>
+    <t>遮挡物没有完全挡住目标，遮挡物在遮挡目标时变成了透明的</t>
+  </si>
+  <si>
+    <t>方块、球体→方块被遮住、球体异常显现在挡板表面</t>
   </si>
 </sst>
 </file>
@@ -1680,7 +1698,7 @@
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="0.0&quot; 秒（约）&quot;"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -1708,7 +1726,7 @@
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1716,14 +1734,14 @@
       <sz val="11"/>
       <color rgb="FF800080"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1739,7 +1757,7 @@
       <sz val="11"/>
       <color rgb="FF7F7F7F"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1770,7 +1788,7 @@
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1778,7 +1796,7 @@
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1786,7 +1804,7 @@
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1794,14 +1812,14 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1809,42 +1827,35 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C6500"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -1911,19 +1922,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
+        <fgColor theme="4" tint="0.79998"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
+        <fgColor theme="4" tint="0.59999"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
+        <fgColor theme="4" tint="0.39998"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1935,19 +1946,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
+        <fgColor theme="5" tint="0.79998"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
+        <fgColor theme="5" tint="0.59999"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
+        <fgColor theme="5" tint="0.39998"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1959,19 +1970,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
+        <fgColor theme="6" tint="0.79998"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
+        <fgColor theme="6" tint="0.59999"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
+        <fgColor theme="6" tint="0.39998"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1983,19 +1994,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
+        <fgColor theme="7" tint="0.79998"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
+        <fgColor theme="7" tint="0.59999"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
+        <fgColor theme="7" tint="0.39998"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2007,19 +2018,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor theme="8" tint="0.79998"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
+        <fgColor theme="8" tint="0.59999"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
+        <fgColor theme="8" tint="0.39998"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2031,19 +2042,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor theme="9" tint="0.79998"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
+        <fgColor theme="9" tint="0.59999"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor theme="9" tint="0.39998"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2085,7 +2096,7 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+        <color theme="4" tint="0.49998"/>
       </bottom>
       <diagonal/>
     </border>
@@ -2234,10 +2245,10 @@
     <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2246,10 +2257,10 @@
     <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2258,10 +2269,10 @@
     <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2270,10 +2281,10 @@
     <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2282,10 +2293,10 @@
     <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2294,10 +2305,10 @@
     <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2305,7 +2316,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2327,6 +2338,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="50">
@@ -2809,7 +2823,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J250"/>
+  <dimension ref="A1:J252"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -8597,6 +8611,52 @@
         <v>11</v>
       </c>
     </row>
+    <row r="251" ht="64" customHeight="1" spans="1:7">
+      <c r="A251" s="3" t="s">
+        <v>551</v>
+      </c>
+      <c r="B251" s="3">
+        <v>2</v>
+      </c>
+      <c r="C251" s="8" t="s">
+        <v>552</v>
+      </c>
+      <c r="D251" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="E251" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="F251" s="5">
+        <v>2.7</v>
+      </c>
+      <c r="G251" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="252" ht="64" customHeight="1" spans="1:7">
+      <c r="A252" s="3" t="s">
+        <v>554</v>
+      </c>
+      <c r="B252" s="3">
+        <v>2</v>
+      </c>
+      <c r="C252" s="8" t="s">
+        <v>555</v>
+      </c>
+      <c r="D252" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="E252" s="4" t="s">
+        <v>556</v>
+      </c>
+      <c r="F252" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="G252" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="B2:B250">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">

</xml_diff>